<commit_message>
Fix Followers/Likes columns to plain text for Google Sheets conversion
Google's xlsx-to-Sheets auto-conversion was rejecting the file with
"Invalid conversion requested" whenever a Followers/Likes column mixed
numeric and text ("n/a") values. Casting both columns to strings fixed it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KSZnuekHgBrAnsDiYAiQb4
</commit_message>
<xml_diff>
--- a/nh_creator_scout/NH_TikTok_Scout_AgeFormat.xlsx
+++ b/nh_creator_scout/NH_TikTok_Scout_AgeFormat.xlsx
@@ -556,11 +556,15 @@
           <t>@econabdallah</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>178100</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>947900</v>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>178100</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>947900</t>
+        </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -937,8 +941,10 @@
           <t>@deserttrader6906</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>52000</v>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>52000</t>
+        </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -990,8 +996,10 @@
           <t>@assadalsharef</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>1100000</v>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>1100000</t>
+        </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -1208,8 +1216,10 @@
           <t>@abo_ahmed_al3mda</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>11900</v>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>11900</t>
+        </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1316,11 +1326,15 @@
           <t>@jubail_aqari</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>33500</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>165900</v>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>33500</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>165900</t>
+        </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -1367,11 +1381,15 @@
           <t>@aqarapp</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
-        <v>99800</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>362700</v>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>99800</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>362700</t>
+        </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1473,11 +1491,15 @@
           <t>@rr05l</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
-        <v>37000</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>1500000</v>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>37000</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>1500000</t>
+        </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 5 stricter-qualified replacement TikTok creators (25 total)
A follow-up research pass under a stricter bar (real named individual only,
independently-confirmed Saudi nationality, corroborating source beyond the
TikTok page itself) found 2 trading and 3 real-estate candidates. No new
e-commerce candidates cleared the bar this round.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KSZnuekHgBrAnsDiYAiQb4
</commit_message>
<xml_diff>
--- a/nh_creator_scout/NH_TikTok_Scout_AgeFormat.xlsx
+++ b/nh_creator_scout/NH_TikTok_Scout_AgeFormat.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1624,6 +1624,281 @@
       <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Real-estate news/commentary niche | Low confidence — handle cluster needs manual disambiguation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>رعد الحربي (أبو دانه)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Raad Al-Harbi ("Abu Danah")</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@abu_danah00</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>@abu_danah00</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>n/a — not visually verified (TikTok inaccessible in this research environment)</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED — could not view TikTok videos directly (blocked in this environment)</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Named individual (tribal surname Al-Harbi) with self-declared Saudi flag; cross-verified via 3 independent properties beyond the TikTok page (X, YouTube, own academy site); risk-aware framing, not signal-selling</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>محمد الخضير</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Mohammed Alkhudhair</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@mohakhuu</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>@mohakhuu</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>114000</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>n/a — not visually verified (TikTok inaccessible in this research environment)</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED — could not view TikTok videos directly (blocked in this environment)</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Named individual with a disclosed, non-hype comparison methodology; strongly Saudi-contextualized content (PIF, Saudia Airlines, Saudi banks, CMA-licensed apps); cross-verified via X + Instagram under consistent name/photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>عماد منشي</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Emad Munshi</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@emad_munshi</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>@emad_munshi</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>165700</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>543300</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>n/a — not visually verified (TikTok inaccessible in this research environment)</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED — could not view TikTok videos directly (blocked in this environment)</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Named individual with a consistent identity across TikTok/X/Instagram/Snapchat/website; explicit Jeddah, Saudi tie via his company, independently confirmed beyond the TikTok page</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>سعد بن محمد التويم</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Saad bin Mohammed Al-Tuwaim</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@saadaltwaim1</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>@saadaltwaim1</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>133200</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>490100</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>n/a — not visually verified (TikTok inaccessible in this research environment)</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED — could not view TikTok videos directly (blocked in this environment)</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Real named individual with a documented corporate role (Tathmen chairman), independently confirmed via the company's own site and 4 distinct platforms (X, YouTube, Facebook, LinkedIn) under a consistent name</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>طارق شقرون</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Tariq Shagroon ("Mr. Broker")</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@tshagroon</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>@tshagroon</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>194800</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>n/a — not visually verified (TikTok inaccessible in this research environment)</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED — could not view TikTok videos directly (blocked in this environment)</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Named individual (not a brand/listings account); explicit Madinah tie across content and company; independently corroborated by two separate news/feature articles plus a distinct company website</t>
         </is>
       </c>
     </row>
@@ -1649,6 +1924,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>